<commit_message>
deploy: main → 374071b88c8009e50dee2eedeeb59c5191e45b2c
</commit_message>
<xml_diff>
--- a/StructureDefinition-alert-asserter.xlsx
+++ b/StructureDefinition-alert-asserter.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-02T11:47:48+00:00</t>
+    <t>2026-10-06T07:04:04+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -331,7 +331,7 @@
     <t>Extension.value[x]</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(PractitionerRole)
+    <t xml:space="preserve">Reference(https://fhir.inera.se/ig/ehds-tk/StructureDefinition/SEEHDSPractitionerRole)
 </t>
   </si>
   <si>
@@ -665,7 +665,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="22.69921875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="68.515625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>